<commit_message>
Reorganise columns according to Gov ID Finder expectations
</commit_message>
<xml_diff>
--- a/data/xlsx/BR.xlsx
+++ b/data/xlsx/BR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mark/sites/codeforiati/gov-id-finder-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F8BF653-F5BC-3C4E-A53B-BB1132F84E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768DB54E-C0A2-9F4B-8F35-B3C731A0BE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="37160" yWindow="880" windowWidth="27640" windowHeight="16680" xr2:uid="{DC1A7E6E-3EF1-8842-8DF9-86C37FD0F6E8}"/>
   </bookViews>
@@ -750,9 +750,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -792,13 +791,13 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{EC632132-3383-5F4F-8195-FDFF3BEA17DF}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="6">
+  <queryTableRefresh nextId="8">
     <queryTableFields count="5">
+      <queryTableField id="2" name="Code" tableColumnId="2"/>
+      <queryTableField id="4" name="Name (English)" tableColumnId="4"/>
+      <queryTableField id="3" name="Name (Portuguese)" tableColumnId="3"/>
+      <queryTableField id="5" name="Branch / Sector" tableColumnId="5"/>
       <queryTableField id="1" name="Identifier" tableColumnId="1"/>
-      <queryTableField id="2" name="Code" tableColumnId="2"/>
-      <queryTableField id="3" name="Name (Portuguese)" tableColumnId="3"/>
-      <queryTableField id="4" name="Name (English)" tableColumnId="4"/>
-      <queryTableField id="5" name="Branch / Sector" tableColumnId="5"/>
     </queryTableFields>
   </queryTableRefresh>
 </queryTable>
@@ -819,11 +818,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{50A00402-D64B-0148-9096-1D1400E3AA39}" name="BR_COA" displayName="BR_COA" ref="A1:E57" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E57" xr:uid="{50A00402-D64B-0148-9096-1D1400E3AA39}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7221928D-0B71-8746-B094-C337FFBF3DDC}" uniqueName="1" name="Identifier" queryTableFieldId="1" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{96967B17-EEF4-0048-80C7-0D8DA7232DAB}" uniqueName="2" name="code" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{DD916E47-5170-244B-B345-8102FC4FB19C}" uniqueName="3" name="name_pt" queryTableFieldId="3" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{7E00EBF0-5C8E-354E-A397-AE80C8A9E62B}" uniqueName="4" name="name_en" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{FFC89C67-C80B-8441-9767-AEED3A8E8125}" uniqueName="5" name="Branch / Sector" queryTableFieldId="5" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{7E00EBF0-5C8E-354E-A397-AE80C8A9E62B}" uniqueName="4" name="name_en" queryTableFieldId="4" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{DD916E47-5170-244B-B345-8102FC4FB19C}" uniqueName="3" name="name_pt" queryTableFieldId="3" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{FFC89C67-C80B-8441-9767-AEED3A8E8125}" uniqueName="5" name="Branch / Sector" queryTableFieldId="5" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{7221928D-0B71-8746-B094-C337FFBF3DDC}" uniqueName="1" name="Identifier" queryTableFieldId="1" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -833,8 +832,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{18D7C385-C1C6-9142-ADC5-5E4D76D2CB0C}" name="BR_COA_meta" displayName="BR_COA_meta" ref="A1:B19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:B19" xr:uid="{18D7C385-C1C6-9142-ADC5-5E4D76D2CB0C}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{94131F7F-5E04-0F47-951E-F70E60096522}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{74093554-20E5-6B48-B19D-403172F7877C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{94131F7F-5E04-0F47-951E-F70E60096522}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{74093554-20E5-6B48-B19D-403172F7877C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1160,980 +1159,980 @@
   <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="66.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>215</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C1" t="s">
         <v>220</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5">
+        <v>10000</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
         <v>12</v>
       </c>
-      <c r="B5">
-        <v>10000</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="1" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>11000</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="E6" t="s">
         <v>16</v>
       </c>
-      <c r="B6">
-        <v>11000</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>12000</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="E7" t="s">
         <v>19</v>
       </c>
-      <c r="B7">
-        <v>12000</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>13000</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="B8">
-        <v>13000</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>14000</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="E9" t="s">
         <v>25</v>
       </c>
-      <c r="B9">
-        <v>14000</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="1" t="s">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>15000</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="E10" t="s">
         <v>28</v>
       </c>
-      <c r="B10">
-        <v>15000</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="1" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>16000</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="E11" t="s">
         <v>31</v>
       </c>
-      <c r="B11">
-        <v>16000</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="1" t="s">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>17000</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="E12" t="s">
         <v>34</v>
       </c>
-      <c r="B12">
-        <v>17000</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13">
+        <v>29000</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" t="s">
         <v>37</v>
       </c>
-      <c r="B13">
-        <v>29000</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="1" t="s">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>34000</v>
+      </c>
+      <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="E14" t="s">
         <v>41</v>
       </c>
-      <c r="B14">
-        <v>34000</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="1" t="s">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>59000</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="E15" t="s">
         <v>44</v>
       </c>
-      <c r="B15">
-        <v>59000</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="1" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>63000</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="B16">
-        <v>63000</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17">
+        <v>20000</v>
+      </c>
+      <c r="B17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E17" t="s">
         <v>50</v>
       </c>
-      <c r="B17">
-        <v>20000</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" s="1" t="s">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>37000</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="E18" t="s">
         <v>54</v>
       </c>
-      <c r="B18">
-        <v>37000</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E18" s="1" t="s">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>60000</v>
+      </c>
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="E19" t="s">
         <v>57</v>
       </c>
-      <c r="B19">
-        <v>60000</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+      <c r="A20">
+        <v>22000</v>
+      </c>
+      <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" t="s">
         <v>60</v>
       </c>
-      <c r="B20">
-        <v>22000</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
+      <c r="A21">
+        <v>24000</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" t="s">
         <v>64</v>
       </c>
-      <c r="B21">
-        <v>24000</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
+      <c r="A22">
+        <v>25000</v>
+      </c>
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" t="s">
         <v>67</v>
       </c>
-      <c r="B22">
-        <v>25000</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
+      <c r="A23">
+        <v>26000</v>
+      </c>
+      <c r="B23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" t="s">
         <v>70</v>
       </c>
-      <c r="B23">
-        <v>26000</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
+      <c r="A24">
+        <v>28000</v>
+      </c>
+      <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" t="s">
         <v>73</v>
       </c>
-      <c r="B24">
-        <v>28000</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
+      <c r="A25">
+        <v>30000</v>
+      </c>
+      <c r="B25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" t="s">
         <v>76</v>
       </c>
-      <c r="B25">
-        <v>30000</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+      <c r="A26">
+        <v>32000</v>
+      </c>
+      <c r="B26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" t="s">
+        <v>63</v>
+      </c>
+      <c r="E26" t="s">
         <v>79</v>
       </c>
-      <c r="B26">
-        <v>32000</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
+      <c r="A27">
+        <v>33000</v>
+      </c>
+      <c r="B27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" t="s">
         <v>82</v>
       </c>
-      <c r="B27">
-        <v>33000</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
+      <c r="A28">
+        <v>35000</v>
+      </c>
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" t="s">
+        <v>63</v>
+      </c>
+      <c r="E28" t="s">
         <v>85</v>
       </c>
-      <c r="B28">
-        <v>35000</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+      <c r="A29">
+        <v>36000</v>
+      </c>
+      <c r="B29" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" t="s">
         <v>88</v>
       </c>
-      <c r="B29">
-        <v>36000</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
+      <c r="A30">
+        <v>38000</v>
+      </c>
+      <c r="B30" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D30" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" t="s">
         <v>91</v>
       </c>
-      <c r="B30">
-        <v>38000</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
+      <c r="A31">
+        <v>39000</v>
+      </c>
+      <c r="B31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" t="s">
         <v>94</v>
       </c>
-      <c r="B31">
-        <v>39000</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
+      <c r="A32">
+        <v>41000</v>
+      </c>
+      <c r="B32" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" t="s">
         <v>97</v>
       </c>
-      <c r="B32">
-        <v>41000</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
+      <c r="A33">
+        <v>42000</v>
+      </c>
+      <c r="B33" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" t="s">
         <v>100</v>
       </c>
-      <c r="B33">
-        <v>42000</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
+      <c r="A34">
+        <v>44000</v>
+      </c>
+      <c r="B34" t="s">
+        <v>105</v>
+      </c>
+      <c r="C34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E34" t="s">
         <v>103</v>
       </c>
-      <c r="B34">
-        <v>44000</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
+      <c r="A35">
+        <v>46000</v>
+      </c>
+      <c r="B35" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" t="s">
         <v>106</v>
       </c>
-      <c r="B35">
-        <v>46000</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
+      <c r="A36">
+        <v>47000</v>
+      </c>
+      <c r="B36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C36" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" t="s">
+        <v>63</v>
+      </c>
+      <c r="E36" t="s">
         <v>109</v>
       </c>
-      <c r="B36">
-        <v>47000</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+      <c r="A37">
+        <v>49000</v>
+      </c>
+      <c r="B37" t="s">
+        <v>114</v>
+      </c>
+      <c r="C37" t="s">
+        <v>113</v>
+      </c>
+      <c r="D37" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" t="s">
         <v>112</v>
       </c>
-      <c r="B37">
-        <v>49000</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+      <c r="A38">
+        <v>51000</v>
+      </c>
+      <c r="B38" t="s">
+        <v>117</v>
+      </c>
+      <c r="C38" t="s">
+        <v>116</v>
+      </c>
+      <c r="D38" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" t="s">
         <v>115</v>
       </c>
-      <c r="B38">
-        <v>51000</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
+      <c r="A39">
+        <v>52000</v>
+      </c>
+      <c r="B39" t="s">
+        <v>120</v>
+      </c>
+      <c r="C39" t="s">
+        <v>119</v>
+      </c>
+      <c r="D39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" t="s">
         <v>118</v>
       </c>
-      <c r="B39">
-        <v>52000</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
+      <c r="A40">
+        <v>53000</v>
+      </c>
+      <c r="B40" t="s">
+        <v>123</v>
+      </c>
+      <c r="C40" t="s">
+        <v>122</v>
+      </c>
+      <c r="D40" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" t="s">
         <v>121</v>
       </c>
-      <c r="B40">
-        <v>53000</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+      <c r="A41">
+        <v>54000</v>
+      </c>
+      <c r="B41" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" t="s">
+        <v>63</v>
+      </c>
+      <c r="E41" t="s">
         <v>124</v>
       </c>
-      <c r="B41">
-        <v>54000</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="A42">
+        <v>55000</v>
+      </c>
+      <c r="B42" t="s">
+        <v>129</v>
+      </c>
+      <c r="C42" t="s">
+        <v>128</v>
+      </c>
+      <c r="D42" t="s">
+        <v>63</v>
+      </c>
+      <c r="E42" t="s">
         <v>127</v>
       </c>
-      <c r="B42">
-        <v>55000</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
+      <c r="A43">
+        <v>56000</v>
+      </c>
+      <c r="B43" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" t="s">
+        <v>131</v>
+      </c>
+      <c r="D43" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" t="s">
         <v>130</v>
       </c>
-      <c r="B43">
-        <v>56000</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
+      <c r="A44">
+        <v>58000</v>
+      </c>
+      <c r="B44" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" t="s">
+        <v>134</v>
+      </c>
+      <c r="D44" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" t="s">
         <v>133</v>
       </c>
-      <c r="B44">
-        <v>58000</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+      <c r="A45">
+        <v>65000</v>
+      </c>
+      <c r="B45" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" t="s">
+        <v>137</v>
+      </c>
+      <c r="D45" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" t="s">
         <v>136</v>
       </c>
-      <c r="B45">
-        <v>65000</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="1" t="s">
+      <c r="A46">
+        <v>67000</v>
+      </c>
+      <c r="B46" t="s">
+        <v>141</v>
+      </c>
+      <c r="C46" t="s">
+        <v>140</v>
+      </c>
+      <c r="D46" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46" t="s">
         <v>139</v>
       </c>
-      <c r="B46">
-        <v>67000</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
+      <c r="A47">
+        <v>68000</v>
+      </c>
+      <c r="B47" t="s">
+        <v>144</v>
+      </c>
+      <c r="C47" t="s">
+        <v>143</v>
+      </c>
+      <c r="D47" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" t="s">
         <v>142</v>
       </c>
-      <c r="B47">
-        <v>68000</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="A48">
+        <v>69000</v>
+      </c>
+      <c r="B48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C48" t="s">
+        <v>146</v>
+      </c>
+      <c r="D48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" t="s">
         <v>145</v>
       </c>
-      <c r="B48">
-        <v>69000</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
+      <c r="A49">
+        <v>81000</v>
+      </c>
+      <c r="B49" t="s">
+        <v>150</v>
+      </c>
+      <c r="C49" t="s">
+        <v>149</v>
+      </c>
+      <c r="D49" t="s">
+        <v>63</v>
+      </c>
+      <c r="E49" t="s">
         <v>148</v>
       </c>
-      <c r="B49">
-        <v>81000</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
+      <c r="A50">
+        <v>82000</v>
+      </c>
+      <c r="B50" t="s">
+        <v>153</v>
+      </c>
+      <c r="C50" t="s">
+        <v>152</v>
+      </c>
+      <c r="D50" t="s">
+        <v>63</v>
+      </c>
+      <c r="E50" t="s">
         <v>151</v>
       </c>
-      <c r="B50">
-        <v>82000</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
+      <c r="A51">
+        <v>84000</v>
+      </c>
+      <c r="B51" t="s">
+        <v>156</v>
+      </c>
+      <c r="C51" t="s">
+        <v>155</v>
+      </c>
+      <c r="D51" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" t="s">
         <v>154</v>
       </c>
-      <c r="B51">
-        <v>84000</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
+      <c r="A52">
+        <v>25201</v>
+      </c>
+      <c r="B52" t="s">
+        <v>159</v>
+      </c>
+      <c r="C52" t="s">
+        <v>158</v>
+      </c>
+      <c r="D52" t="s">
+        <v>160</v>
+      </c>
+      <c r="E52" t="s">
         <v>157</v>
       </c>
-      <c r="B52">
-        <v>25201</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="1" t="s">
+      <c r="A53">
+        <v>71000</v>
+      </c>
+      <c r="B53" t="s">
+        <v>163</v>
+      </c>
+      <c r="C53" t="s">
+        <v>162</v>
+      </c>
+      <c r="D53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E53" t="s">
         <v>161</v>
       </c>
-      <c r="B53">
-        <v>71000</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E53" s="1" t="s">
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>73000</v>
+      </c>
+      <c r="B54" t="s">
+        <v>167</v>
+      </c>
+      <c r="C54" t="s">
+        <v>166</v>
+      </c>
+      <c r="D54" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
+      <c r="E54" t="s">
         <v>165</v>
       </c>
-      <c r="B54">
-        <v>73000</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E54" s="1" t="s">
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>74000</v>
+      </c>
+      <c r="B55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C55" t="s">
+        <v>169</v>
+      </c>
+      <c r="D55" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
+      <c r="E55" t="s">
         <v>168</v>
       </c>
-      <c r="B55">
-        <v>74000</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="E55" s="1" t="s">
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>75000</v>
+      </c>
+      <c r="B56" t="s">
+        <v>173</v>
+      </c>
+      <c r="C56" t="s">
+        <v>172</v>
+      </c>
+      <c r="D56" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
+      <c r="E56" t="s">
         <v>171</v>
       </c>
-      <c r="B56">
-        <v>75000</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="E56" s="1" t="s">
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>90000</v>
+      </c>
+      <c r="B57" t="s">
+        <v>176</v>
+      </c>
+      <c r="C57" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
+      <c r="E57" t="s">
         <v>174</v>
-      </c>
-      <c r="B57">
-        <v>90000</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -2162,146 +2161,146 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>179</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>181</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>183</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>185</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>187</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>189</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>191</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>193</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>195</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>199</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>201</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>203</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>205</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>207</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>209</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>211</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>213</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>214</v>
       </c>
     </row>

</xml_diff>